<commit_message>
Rewrite brand-mention replies as plain suggestions for a Lynkk-labelled account
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015dXgfxu1ugCxsD9bCGxkqs
</commit_message>
<xml_diff>
--- a/lynkk-reddit-leads/results/2026-10-11/all_items_with_links_2026-10-11.xlsx
+++ b/lynkk-reddit-leads/results/2026-10-11/all_items_with_links_2026-10-11.xlsx
@@ -619,8 +619,8 @@
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>Depends a lot on where your in-person meetings happen. If there's usually a laptop on the table anyway, I'd try recording from that before buying a Plaud or Pocket. A laptop mic is fine for a small room, and you end up with everything in one app instead of two, which you'll appreciate when you're looking for something from three weeks ago. A recorder makes more sense if you're often in cafes or on site.
-Full disclosure, I work on Lynkk, which does that combo (calls without a bot, in-person from the browser), so I'm biased. But the one-place thing matters whichever tool you pick.</t>
+          <t>Depends on where your in-person meetings happen. If there's usually a laptop on the table, try recording from that before buying a Plaud or Pocket; a laptop mic is fine for a small room, and you get everything in one app instead of two. A recorder makes more sense for cafes or site visits.
+If you want one tool for both, Lynkk is worth a look: it records Zoom, Meet and Teams calls without a bot joining, and in-person meetings straight from the browser, so it all ends up searchable in one place.</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -710,9 +710,8 @@
       </c>
       <c r="P3" s="3" t="inlineStr">
         <is>
-          <t>The weeks-later gap is the real test, and most demos never show it. Record a consult, don't touch it for two weeks, then try to draft from the notes alone and see what's missing. Day-one summaries all look fine.
-Also +1 on a cheap boundary mic for in-person, it matters more than the app.
-I'm on the Lynkk team, so grain of salt, but if you want a software-only option to compare against Plaud Desktop, it records in the browser for in-person and through a Mac app for calls, and every point in the notes links back to the spot in the recording. Worth running the same consult through both.</t>
+          <t>The weeks-later gap is the real test, and demos never show it. Record a consult, leave it for two weeks, then try to draft from the notes alone and see what's missing. A cheap boundary mic on the table also matters more than the app for in-person.
+For a software-only comparison against Plaud Desktop, Lynkk is one to try: it records in-person consults in the browser and video calls through a Mac app, and every point in the notes links back to the exact spot in the recording, which helps when you're drafting weeks later.</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -802,8 +801,8 @@
       </c>
       <c r="P4" s="3" t="inlineStr">
         <is>
-          <t>Phone calls are the annoying one. Almost nothing can record a regular iPhone call, so people either take important calls on the laptop (FaceTime or WhatsApp desktop) or live with a separate app for those.
-Zoom plus in-person in one place is the easy part. Disclosure, I work on Lynkk, which handles those two and keeps them searchable together, but there's no phone app, so it wouldn't fix the iPhone bit. Whatever you go with, I'd rank 'one place to search' above anything else on the feature list.</t>
+          <t>Phone calls are the hard part. Almost nothing can record a regular iPhone call, so the usual workaround is taking important calls on the laptop through FaceTime or WhatsApp desktop.
+For Zoom plus in-person in one place, Lynkk covers both: the Mac app picks up Zoom, Meet, Teams, FaceTime and WhatsApp calls without a bot, and in-person meetings can be recorded from the browser, all searchable together. No phone app though, so native iPhone calls stay the gap.</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -893,8 +892,8 @@
       </c>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>This is the thing summaries are worst at, because each one only knows its own meeting. What tends to work better is asking across the whole project ('what's the current launch date and when did it change?') and only trusting answers that point to the specific meeting and moment, so you can click through and see whether it was a real decision or just someone floating it.
-Disclosure, I work on Lynkk, and that's roughly how its chat works: answers from your own notes, with citations you can click. Not a proper decision timeline though. Would love to see someone build that.</t>
+          <t>Summaries are bad at this because each one only knows its own meeting. What works better is asking across the whole project ('what's the current launch date and when did it change?') and only trusting answers that point to the specific meeting and moment, so you can check whether it was a real decision or just someone floating an idea.
+Lynkk's chat works roughly that way: it answers only from your own notes, finds them by project, and every answer has citations that open the note at the exact moment. Not a dedicated decision timeline, but it handles the 'what's current and why' question.</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -984,8 +983,8 @@
       </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>Copilot's fine for internal stuff, but it really only covers meetings your tenant hosts, so customer calls on their Zoom links fall through. For the budget conversation I'd count how many important customer calls last month were outside Teams. That number usually settles it.
-If you do add something, look for one that records from the laptop instead of joining as a bot, then it doesn't matter whose link it is. (I work on Lynkk, which works that way on Mac, so yes, biased. Apple silicon only though.)</t>
+          <t>Copilot only really covers meetings your tenant hosts, so customer calls on their Zoom links fall through. For the budget conversation, count how many important customer calls last month were outside Teams; that number usually settles it.
+If you add something, pick a tool that records from the laptop instead of joining as a bot, so it doesn't matter whose link it is. Lynkk's Mac app works like that across Zoom, Meet, Teams and Webex (Apple silicon Macs only).</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -1075,8 +1074,8 @@
       </c>
       <c r="P7" s="3" t="inlineStr">
         <is>
-          <t>If customers are fine with recording, I'd skip the tablet and handwriting route. You'd still be summarizing your own notes afterwards. Record the meeting, let the tool pull the next steps, and the follow-up email is mostly done.
-Salesforce is where most of these tools get vague, so ask straight out whether it updates fields or just hands you text. Disclosure: I work on Lynkk, which covers the record and next steps part from a laptop, but it doesn't sync to Salesforce, so that bit would stay manual.</t>
+          <t>If customers are fine with recording, skip the tablet and handwriting route; you'd still be summarizing your own notes afterwards. Record the meeting, let the tool pull out next steps, and the follow-up email is mostly written.
+For in-person meetings from a laptop, Lynkk records in the browser and gives you decisions and action items with owners and due dates. It doesn't sync to Salesforce, so check that part with any tool you try, since most only hand you text.</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -1166,8 +1165,8 @@
       </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
-          <t>The thing that breaks in practice is external Zoom calls where the host's settings hold bots in the waiting room. So whatever you pick, make sure it can also record from the user's own machine as a fallback. Then run a two-week pilot with whoever lives on Zoom and just count how many external calls actually got captured.
-I'm on the Lynkk team, bias noted. It has a bot for Teams, Zoom and Meet plus a no-bot Mac app and Chrome extension for the blocked cases, all in one archive. Workspaces cap at 10 seats though, so only relevant if this client's team is small.</t>
+          <t>What usually breaks is external Zoom calls where the host's settings hold bots in the waiting room, so make sure whatever you pick can also record from the user's own machine. Then pilot it for two weeks with the heaviest Zoom users and count how many external calls actually got captured.
+Lynkk handles both cases in one archive: a bot for Teams, Zoom and Meet, plus a no-bot Mac app and Chrome extension for when bots get blocked. Workspaces cap at 10 seats, so it only fits a small team.</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -1257,8 +1256,8 @@
       </c>
       <c r="P9" s="3" t="inlineStr">
         <is>
-          <t>The biggest difference on long meetings is whether you can jump from a line in the summary straight to that moment in the audio. Saves so much scrubbing. And test with a real 90 minute meeting, not a 10 minute demo; that's where summaries start getting mushy.
-(Disclosure: I work on Lynkk, which does the timestamp-to-audio thing, but it's Mac, Chrome and web, not a pocket recorder, so it's a different setup from Plaud.)</t>
+          <t>The biggest difference on long meetings is whether you can jump from a line in the summary straight to that moment in the audio; it saves a lot of scrubbing. Test with a real 90-minute meeting, not a short demo, because that's where summaries go vague.
+Lynkk does the timestamp-to-audio part well: every takeaway plays the recording from that moment. It's Mac, Chrome and web rather than a pocket recorder, so it's a different setup from Plaud.</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -1348,8 +1347,8 @@
       </c>
       <c r="P10" s="3" t="inlineStr">
         <is>
-          <t>You'll probably always do some review, but it can be a two-minute skim instead of a reread. What cuts it down most is when every action item has a timestamp you can click to hear the original moment, so you only check the ones that look off. Saying owners and dates out loud at the end of the call helps a ton too.
-Disclosure, I work on Lynkk, which is built around that click-to-check idea. Honestly though, the verbal recap at the end helps with any tool.</t>
+          <t>Some review will always be needed, but it can be a two-minute skim. What cuts it down most is every action item having a timestamp you can click to hear the original moment, so you only check the ones that look off. Saying owners and dates out loud at the end of the call helps a lot too.
+Lynkk is built around that click-to-check idea: decisions, action items with owners and due dates, and open questions, each linked back to the recording.</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -1439,8 +1438,8 @@
       </c>
       <c r="P11" s="3" t="inlineStr">
         <is>
-          <t>That 'inferred urgency' thing is exactly why action items need a source. Simplest rule: every action item links to the moment it was said, and anything without a source stays a draft. That catches invented deadlines in seconds. Also have owners confirm their own items instead of the PM approving everything.
-Disclosure, I work on Lynkk. Its action items each carry a timestamp back to the recording, and nothing goes to Jira unless someone sends it by hand.</t>
+          <t>That 'inferred urgency' is why action items need a source. Simplest rule: every action item links to the moment it was said, and anything without a source stays a draft. That catches invented deadlines in seconds. Also have owners confirm their own items instead of the PM approving everything.
+Lynkk works this way: each action item carries a timestamp back to the recording, and nothing goes to Jira unless someone sends it by hand.</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -1530,8 +1529,8 @@
       </c>
       <c r="P12" s="3" t="inlineStr">
         <is>
-          <t>Depends whether you need the meeting data inside your own agent or just need answers. If it's mostly 'what did we decide with X' and 'what's still open', asking inside the notes tool is simpler than wiring transcripts into an agent. If the agent needs to act on it alongside other context, then yeah, your MCP route makes sense.
-I work on Lynkk so I'm biased, but it's the first kind: you ask across your notes, get answers that link back to the moment, and can create a Jira issue from there. Not sure it fits if you need it inside your own agent.</t>
+          <t>Depends whether you need the meeting data inside your own agent or just need answers. If it's mostly 'what did we decide with X' and 'what's still open', asking inside the notes tool is simpler than wiring transcripts into an agent. If the agent has to act on it with other context, your MCP route makes sense.
+For the first case, Lynkk lets you ask across all your notes, gives answers that link back to the moment, and can create a Jira issue from there. You can ask it from Slack too.</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -1621,8 +1620,8 @@
       </c>
       <c r="P13" s="3" t="inlineStr">
         <is>
-          <t>Checking is the right call. What makes it workable is being able to click a line in the summary and hear the original moment, so checking a detail takes seconds instead of rereading the transcript. Small details are exactly where summaries slip, so I'd trust the summary for the gist and the recording for names and numbers.
-(I work on Lynkk, so bias disclosed. It does the click-to-hear thing, plus search across all your meetings afterwards.)</t>
+          <t>Checking is the right instinct. What makes it workable is clicking a line in the summary and hearing the original moment, so a detail takes seconds to verify instead of rereading the transcript. Trust the summary for the gist and the recording for names and numbers.
+Lynkk does the click-to-hear part: every takeaway and action item has a timestamp that plays the recording, and you can search across all your meetings afterwards.</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -1704,7 +1703,8 @@
       </c>
       <c r="P14" s="3" t="inlineStr">
         <is>
-          <t>Mostly depends on whether you have in-person meetings too. If you do, keep everything in one tool, otherwise you end up searching two places later. I'm on the Lynkk team, which does calls without a bot plus in-person from the browser, but I'd give the same advice for any tool.</t>
+          <t>Mostly depends on whether you have in-person meetings too. If you do, keep everything in one tool, otherwise you end up searching two places later.
+Lynkk is one that covers both: calls without a bot from a Mac app or Chrome extension, and in-person meetings from the browser.</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -1790,7 +1790,8 @@
       </c>
       <c r="P15" s="3" t="inlineStr">
         <is>
-          <t>Totally fair worry. Whatever you pick, export your recordings regularly so you're never stuck, and do a short side-by-side with a second tool before recommending anything firm-wide. (I work on Lynkk, so I'm one of the options. It's software only, so there's no hardware to bet on.)</t>
+          <t>Fair worry. Whatever you pick, export your recordings regularly so you're never stuck, and do a short side-by-side with a second tool before recommending anything firm-wide.
+If you want a software-only option to compare, Lynkk is one: no hardware to bet on, in-person recording from the browser, and calls through a Mac app.</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -1876,7 +1877,8 @@
       </c>
       <c r="P16" s="3" t="inlineStr">
         <is>
-          <t>Attendee-only is a good guardrail, but I'd go one step further: only set an owner when someone actually said it, with a link to that moment. Otherwise mark it 'owner needed'. A 30-second recap at the end ('Priya has the roadmap, Friday') removes most of the guessing. (Disclosure: I work on Lynkk, where every action item links back to the recording, which makes checking this pretty quick.)</t>
+          <t>Attendee-only is a good guardrail, but go one step further: only set an owner when someone actually said it, with a link to that moment, and otherwise mark it 'owner needed'. A 30-second recap at the end ('Priya has the roadmap, Friday') removes most of the guessing.
+Tools that link each action item to the recording make this quick to check; Lynkk does that for every action item.</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -2148,7 +2150,8 @@
       </c>
       <c r="P20" s="3" t="inlineStr">
         <is>
-          <t>Makes sense. If what you need is record, transcribe and summarize reliably, the agent features are just noise. I'd write down the three things you actually rely on and test alternatives against only those. (Biased, I work on Lynkk, which sticks to that core: recording, transcript, and a brief that links back to the audio.)</t>
+          <t>Makes sense. If what you need is record, transcribe and summarize reliably, the agent features are noise. Write down the three things you actually rely on and test alternatives against only those.
+Lynkk is worth adding to that test since it sticks to the core: recording, transcript, and a brief that links back to the audio.</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
@@ -2234,7 +2237,8 @@
       </c>
       <c r="P21" s="3" t="inlineStr">
         <is>
-          <t>Mixed language is rough for most engines. Setting the languages explicitly, if your tool lets you, and adding names and terms to a custom vocab usually helps more than anything. If you want a comparison point, I work on Lynkk, which does 17 languages with auto-detect plus a custom words list. Might be worth one side-by-side on a mixed meeting.</t>
+          <t>Mixed language is rough for most engines. Setting the languages explicitly, if your tool allows it, and adding names and terms to a custom vocabulary usually helps more than anything.
+For a comparison point, Lynkk transcribes 17 languages with auto-detect and has a custom words list. Worth one side-by-side on a mixed meeting.</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
@@ -2320,7 +2324,8 @@
       </c>
       <c r="P22" s="3" t="inlineStr">
         <is>
-          <t>The summary itself rarely saves time. What helps is when 'we could try this' gets filed as an open question instead of a decision, and you can click back to hear how it was actually said. (Disclosure: I work on Lynkk, which records without a bot too. Curious what other people find actually gets opened after the meeting.)</t>
+          <t>The summary itself rarely saves time. What helps is when 'we could try this' gets filed as an open question instead of a decision, and you can click back to hear how it was actually said.
+Lynkk splits decisions, action items and open questions that way and records without a bot, similar to what you like about Bluedot. Curious what others find actually gets opened after the meeting.</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -2406,7 +2411,8 @@
       </c>
       <c r="P23" s="3" t="inlineStr">
         <is>
-          <t>I'd start smaller than a coaching platform. Take five lost deals and five won ones and only listen from the first price mention onward. Patterns show up faster than you'd think. (I work on Lynkk. It's not a coaching tool, but its timestamps let you jump straight to the price discussion instead of replaying the whole hour, which might at least cut the review time.)</t>
+          <t>Start smaller than a coaching platform. Take five lost deals and five won ones and only listen from the first price mention onward; patterns show up faster than you'd expect.
+To cut the listening time, a tool with timestamped takeaways helps you jump straight to the price discussion. Lynkk does that, though it isn't a coaching tool, so it helps with the review time rather than scoring reps.</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">

</xml_diff>